<commit_message>
Auto commit 02-03-2026 14:49:38.63
</commit_message>
<xml_diff>
--- a/Data Base/Global Templates/MWSS with Submersible Pump.xlsx
+++ b/Data Base/Global Templates/MWSS with Submersible Pump.xlsx
@@ -558,7 +558,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -600,7 +600,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2">
-        <v>1</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="29" x14ac:dyDescent="0.25">

</xml_diff>